<commit_message>
Add PIN login, QR hidden missions with score merging, DB-driven events, and team/personal score split
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sheet-template/운동회_시트.xlsx
+++ b/sheet-template/운동회_시트.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -528,141 +528,208 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>설명</t>
+          <t>아이콘</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>모래판 위에서 펼쳐지는 몸싸움 대결!</t>
+          <t>🐷</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>코스마다 주어지는 미션을 클리어하며 달리는 레이스</t>
+          <t>🎯</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>팀 대항 이어달리기</t>
+          <t>🏃</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>팀 대항 피구 대결</t>
+          <t>🏐</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>부리또처럼 몸을 돌돌 감싸고 벌이는 대결</t>
+          <t>🌯</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>발로 하는 야구</t>
+          <t>⚽</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>팀워크로 넘는 단체 줄넘기</t>
+          <t>🪢</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>슬리퍼를 던져 과녁을 맞히는 양궁</t>
+          <t>🩴</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>음악이 멈추면 고깔(의자)을 차지하라</t>
+          <t>🪑</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>이 사람은 누구일까요? 인물 맞히기 퀴즈</t>
+          <t>🧑</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>노래 한 소절 듣고 제목 맞히기</t>
+          <t>🎵</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>히든미션 칩을 스캔해서 완료한 개인 미션</t>
+          <t>🕵️</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
+          <t>설명</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>모래판 위에서 펼쳐지는 몸싸움 대결!</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>코스마다 주어지는 미션을 클리어하며 달리는 레이스 (예: 레몬 먹고 휘파람 불기, 사격으로 캔 넘어뜨리기)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>팀 대항 이어달리기</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>팀 대항 피구 대결</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>부리또처럼 몸을 돌돌 감싸고 벌이는 대결</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>발로 하는 야구</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>팀워크로 넘는 단체 줄넘기</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>슬리퍼를 던져 과녁을 맞히는 양궁</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>음악이 멈추면 고깔(의자)을 차지하라</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>이 사람은 누구일까요? 인물 맞히기 퀴즈</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>노래 한 소절 듣고 제목 맞히기</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>히든미션 칩을 스캔해서 완료한 개인 미션 (점수 기록용 항목)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
           <t>이름</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>이학균</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>김여경</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>홍상웅</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>최연수</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>이재열</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>박지원</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>송효준</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>전주현</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>강이수</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>박시안</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>박종혁</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>황은비</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>※ 종목/이름을 추가·수정할 땐 이 시트만 고치면 다른 시트 드롭다운에 자동 반영됩니다.</t>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>※ 종목/아이콘/설명/이름을 추가·수정할 땐 이 시트만 고치면 앱과 다른 시트 드롭다운에 자동 반영됩니다. (앱은 종목 목록 화면을 이 시트에서 직접 읽어옵니다 — js/data.js는 백엔드 연결 안 됐을 때만 쓰는 예비용입니다)</t>
         </is>
       </c>
     </row>
@@ -677,13 +744,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="90" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -707,6 +777,21 @@
           <t>partner</t>
         </is>
       </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>tier</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>nemesis</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>⚠️ tier(1~3)와 nemesis(그 사람의 라이벌)는 아직 안 채워져 있어요 — 직접 정해서 채워주세요. 히든미션 텍스트의 [티어]/[네메시스]/[파트너]가 이 값들로 치환되어 표시됩니다.</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -729,6 +814,8 @@
           <t>김여경</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -751,6 +838,8 @@
           <t>이학균</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -773,6 +862,8 @@
           <t>최연수</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -795,6 +886,8 @@
           <t>홍상웅</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -817,6 +910,8 @@
           <t>박지원</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -839,6 +934,8 @@
           <t>이재열</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -861,6 +958,8 @@
           <t>전주현</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -883,6 +982,8 @@
           <t>송효준</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -905,6 +1006,8 @@
           <t>박시안</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -927,6 +1030,8 @@
           <t>강이수</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -949,6 +1054,8 @@
           <t>황은비</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -971,11 +1078,13 @@
           <t>박종혁</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="4">
+  <dataValidations count="6">
     <dataValidation sqref="A2:A13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=DB!$B$3:$M$3</formula1>
+      <formula1>=DB!$B$4:$M$4</formula1>
     </dataValidation>
     <dataValidation sqref="B2:B13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"남,여"</formula1>
@@ -984,7 +1093,13 @@
       <formula1>"흑팀,백팀"</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=DB!$B$3:$M$3</formula1>
+      <formula1>=DB!$B$4:$M$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1,2,3"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=DB!$B$4:$M$4</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1139,7 +1254,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="A2:A13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=DB!$B$3:$M$3</formula1>
+      <formula1>=DB!$B$4:$M$4</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1159,7 +1274,7 @@
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="80" customWidth="1" min="6" max="6"/>
+    <col width="90" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1185,14 +1300,14 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>⚠️ 이 시트는 앱에서 본인 것만 필터링되어 보여요(MVP/개인 등수 등). 팀 우승 판정에는 안 씀 — 그건 TeamScoreLog.</t>
+          <t>⚠️ 이 시트는 앱에서 본인 것만 필터링되어 보여요(MVP/개인 등수 등). 팀 우승 판정에는 안 씀 — 그건 TeamScoreLog. '개인미션' event로 시작하는 행은 히든미션 성공 시 onEdit 트리거가 자동으로 추가한 것입니다.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="A2:A151" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=DB!$B$3:$M$3</formula1>
+      <formula1>=DB!$B$4:$M$4</formula1>
     </dataValidation>
     <dataValidation sqref="B2:B151" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=DB!$B$1:$M$1</formula1>
@@ -1264,15 +1379,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="100" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="100" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1288,22 +1404,27 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
+          <t>points</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
           <t>claimedBy</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>claimedAt</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>⚠️ claimedBy/claimedAt/status는 앱이 QR 스캔 시 자동으로 채웁니다(status는 스캔 즉시 '진행중'). 실제로 미션을 해냈는지 확인한 뒤 status를 '성공' 또는 '실패'로 진행자가 직접 바꿔주세요. missionId는 QR코드에 인쇄되는 값이니 바꾸지 마세요.</t>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>⚠️ mission 칸의 [파트너]/[네메시스]/[티어]는 그 칩을 가져간 사람의 Participants 값으로 자동 치환되어 화면에 표시됩니다 (이 시트엔 템플릿 그대로 둡니다). claimedBy/claimedAt/status는 앱이 QR 스캔 시 자동으로 채웁니다(status는 스캔 즉시 '진행중'). 실제로 미션을 해냈는지 확인한 뒤 status를 '성공' 또는 '실패'로 진행자가 직접 바꿔주세요 — '성공'인 칩의 points는 앱이 '내 점수'를 보여줄 때 이 시트에서 실시간으로 읽어와 자동 합산합니다 (따로 옮겨 적을 필요 없고, status를 나중에 정정해도 바로 반영됩니다). missionId는 QR코드에 인쇄되는 값이니 바꾸지 마세요.</t>
         </is>
       </c>
     </row>
@@ -1318,9 +1439,12 @@
           <t>오늘 처음 만난 사람과 하이파이브 5번 하기</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="n">
+        <v>10</v>
+      </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1333,9 +1457,12 @@
           <t>진행자 몰래 셀카 찍고 보여주기</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="n">
+        <v>15</v>
+      </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1345,12 +1472,15 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>처음 만난 사람 이름 외워서 소개하기</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>피구에서 [파트너] 맞춰서 아웃시키기</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>20</v>
+      </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1360,12 +1490,15 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>경기 중 우스꽝스러운 세리머니 하기</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>부리또 듀얼에서 [네메시스] 상대로 승리하기</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>25</v>
+      </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1375,12 +1508,15 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>다른 팀 대놓고 크게 응원해주기</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>발야구에서 [티어]루타 달성하기</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>20</v>
+      </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1390,12 +1526,15 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>오늘 있었던 재밌는 순간 한 줄로 기록하기</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>돼지씨름 [티어]번 이기기</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>20</v>
+      </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1405,12 +1544,15 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>아무나 붙잡고 하이파이브 챌린지 성공시키기</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
+          <t>[네메시스]와 하이파이브하고 화해하기</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>15</v>
+      </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1420,19 +1562,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>본인 소개를 3초 안에 임팩트있게 하기</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
+          <t>[파트너]와 함께 사진찍기</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>10</v>
+      </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="C2:C59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=DB!$B$3:$M$3</formula1>
+    <dataValidation sqref="D2:D59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=DB!$B$4:$M$4</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"진행중,성공,실패"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1503,7 +1648,7 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1519,7 +1664,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>※ 진행자가 개인 시상(MVP 등) 정할 때 참고용. 앱에는 노출되지 않습니다.</t>
+          <t>※ 진행자가 개인 시상(MVP 등) 정할 때 참고용. 앱에는 노출되지 않습니다. PersonalScoreLog 수동 입력분 + MissionChips에서 status가 '성공'인 칩의 points까지 합산됩니다.</t>
         </is>
       </c>
     </row>
@@ -1529,7 +1674,7 @@
         <v/>
       </c>
       <c r="B2">
-        <f>SUMIF(PersonalScoreLog!$A:$A,A2,PersonalScoreLog!$D:$D)</f>
+        <f>SUMIF(PersonalScoreLog!$A:$A,A2,PersonalScoreLog!$D:$D)+SUMIFS(MissionChips!$C:$C,MissionChips!$D:$D,A2,MissionChips!$F:$F,"성공")</f>
         <v/>
       </c>
     </row>
@@ -1539,7 +1684,7 @@
         <v/>
       </c>
       <c r="B3">
-        <f>SUMIF(PersonalScoreLog!$A:$A,A3,PersonalScoreLog!$D:$D)</f>
+        <f>SUMIF(PersonalScoreLog!$A:$A,A3,PersonalScoreLog!$D:$D)+SUMIFS(MissionChips!$C:$C,MissionChips!$D:$D,A3,MissionChips!$F:$F,"성공")</f>
         <v/>
       </c>
     </row>
@@ -1549,7 +1694,7 @@
         <v/>
       </c>
       <c r="B4">
-        <f>SUMIF(PersonalScoreLog!$A:$A,A4,PersonalScoreLog!$D:$D)</f>
+        <f>SUMIF(PersonalScoreLog!$A:$A,A4,PersonalScoreLog!$D:$D)+SUMIFS(MissionChips!$C:$C,MissionChips!$D:$D,A4,MissionChips!$F:$F,"성공")</f>
         <v/>
       </c>
     </row>
@@ -1559,7 +1704,7 @@
         <v/>
       </c>
       <c r="B5">
-        <f>SUMIF(PersonalScoreLog!$A:$A,A5,PersonalScoreLog!$D:$D)</f>
+        <f>SUMIF(PersonalScoreLog!$A:$A,A5,PersonalScoreLog!$D:$D)+SUMIFS(MissionChips!$C:$C,MissionChips!$D:$D,A5,MissionChips!$F:$F,"성공")</f>
         <v/>
       </c>
     </row>
@@ -1569,7 +1714,7 @@
         <v/>
       </c>
       <c r="B6">
-        <f>SUMIF(PersonalScoreLog!$A:$A,A6,PersonalScoreLog!$D:$D)</f>
+        <f>SUMIF(PersonalScoreLog!$A:$A,A6,PersonalScoreLog!$D:$D)+SUMIFS(MissionChips!$C:$C,MissionChips!$D:$D,A6,MissionChips!$F:$F,"성공")</f>
         <v/>
       </c>
     </row>
@@ -1579,7 +1724,7 @@
         <v/>
       </c>
       <c r="B7">
-        <f>SUMIF(PersonalScoreLog!$A:$A,A7,PersonalScoreLog!$D:$D)</f>
+        <f>SUMIF(PersonalScoreLog!$A:$A,A7,PersonalScoreLog!$D:$D)+SUMIFS(MissionChips!$C:$C,MissionChips!$D:$D,A7,MissionChips!$F:$F,"성공")</f>
         <v/>
       </c>
     </row>
@@ -1589,7 +1734,7 @@
         <v/>
       </c>
       <c r="B8">
-        <f>SUMIF(PersonalScoreLog!$A:$A,A8,PersonalScoreLog!$D:$D)</f>
+        <f>SUMIF(PersonalScoreLog!$A:$A,A8,PersonalScoreLog!$D:$D)+SUMIFS(MissionChips!$C:$C,MissionChips!$D:$D,A8,MissionChips!$F:$F,"성공")</f>
         <v/>
       </c>
     </row>
@@ -1599,7 +1744,7 @@
         <v/>
       </c>
       <c r="B9">
-        <f>SUMIF(PersonalScoreLog!$A:$A,A9,PersonalScoreLog!$D:$D)</f>
+        <f>SUMIF(PersonalScoreLog!$A:$A,A9,PersonalScoreLog!$D:$D)+SUMIFS(MissionChips!$C:$C,MissionChips!$D:$D,A9,MissionChips!$F:$F,"성공")</f>
         <v/>
       </c>
     </row>
@@ -1609,7 +1754,7 @@
         <v/>
       </c>
       <c r="B10">
-        <f>SUMIF(PersonalScoreLog!$A:$A,A10,PersonalScoreLog!$D:$D)</f>
+        <f>SUMIF(PersonalScoreLog!$A:$A,A10,PersonalScoreLog!$D:$D)+SUMIFS(MissionChips!$C:$C,MissionChips!$D:$D,A10,MissionChips!$F:$F,"성공")</f>
         <v/>
       </c>
     </row>
@@ -1619,7 +1764,7 @@
         <v/>
       </c>
       <c r="B11">
-        <f>SUMIF(PersonalScoreLog!$A:$A,A11,PersonalScoreLog!$D:$D)</f>
+        <f>SUMIF(PersonalScoreLog!$A:$A,A11,PersonalScoreLog!$D:$D)+SUMIFS(MissionChips!$C:$C,MissionChips!$D:$D,A11,MissionChips!$F:$F,"성공")</f>
         <v/>
       </c>
     </row>
@@ -1629,7 +1774,7 @@
         <v/>
       </c>
       <c r="B12">
-        <f>SUMIF(PersonalScoreLog!$A:$A,A12,PersonalScoreLog!$D:$D)</f>
+        <f>SUMIF(PersonalScoreLog!$A:$A,A12,PersonalScoreLog!$D:$D)+SUMIFS(MissionChips!$C:$C,MissionChips!$D:$D,A12,MissionChips!$F:$F,"성공")</f>
         <v/>
       </c>
     </row>
@@ -1639,7 +1784,7 @@
         <v/>
       </c>
       <c r="B13">
-        <f>SUMIF(PersonalScoreLog!$A:$A,A13,PersonalScoreLog!$D:$D)</f>
+        <f>SUMIF(PersonalScoreLog!$A:$A,A13,PersonalScoreLog!$D:$D)+SUMIFS(MissionChips!$C:$C,MissionChips!$D:$D,A13,MissionChips!$F:$F,"성공")</f>
         <v/>
       </c>
     </row>

</xml_diff>